<commit_message>
chore: update output files
</commit_message>
<xml_diff>
--- a/output/TFL_TOC_v2.1.0.xlsx
+++ b/output/TFL_TOC_v2.1.0.xlsx
@@ -2067,208 +2067,196 @@
       <c r="M26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>F14.2.1</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.2.1</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Forest Plot — Primary Endpoint by Subgroup</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>T14.2.9</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.2.9</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Tumor Response — Best Overall Response (BOR)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADEFF</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>f_forest_primary.sas</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L27" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Oncology only</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADRS</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>t_bor.sas</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>F14.2.2</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.2.2</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Longitudinal Plot — Primary Endpoint Over Time</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>T14.2.10</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.2.10</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Tumor Response — Objective Response Rate (ORR)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADEFF</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>f_longitudinal_eff.sas</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L28" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Oncology only</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADRS</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>t_orr.sas</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>F14.2.3</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.2.3</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Cumulative Distribution Function Plot of Primary Endpoint</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>T14.2.11</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.2.11</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Tumor Response — Disease Control Rate (DCR)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADEFF</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>f_cdf_eff.sas</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="inlineStr"/>
-      <c r="K29" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L29" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M29" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Oncology only</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADRS</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>t_dcr.sas</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>T14.2.9</t>
+          <t>T14.2.12</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.9</t>
+          <t>Table 14.2.12</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Best Overall Response (BOR)</t>
+          <t>Tumor Response — Duration of Response (DOR)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2283,7 +2271,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>Responders (Confirmed CR or PR)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2293,12 +2281,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADRS, ADTTE</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>t_bor.sas</t>
+          <t>t_dor.sas</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -2317,17 +2305,17 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>T14.2.10</t>
+          <t>T14.2.13</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.10</t>
+          <t>Table 14.2.13</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Objective Response Rate (ORR)</t>
+          <t>Tumor Response — Time to Response (TTR)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2342,7 +2330,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>Responders (Confirmed CR or PR)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2357,7 +2345,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>t_orr.sas</t>
+          <t>t_ttr.sas</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -2376,17 +2364,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>T14.2.11</t>
+          <t>T14.2.14</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.11</t>
+          <t>Table 14.2.14</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Disease Control Rate (DCR)</t>
+          <t>Progression-Free Survival (PFS) — Primary Analysis</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2411,12 +2399,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADTTE</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>t_dcr.sas</t>
+          <t>t_pfs_primary.sas</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -2435,17 +2423,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>T14.2.12</t>
+          <t>T14.2.15</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.12</t>
+          <t>Table 14.2.15</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Duration of Response (DOR)</t>
+          <t>Overall Survival (OS) — Primary Analysis</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2460,7 +2448,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Responders (Confirmed CR or PR)</t>
+          <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2470,12 +2458,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS, ADTTE</t>
+          <t>ADSL, ADTTE</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>t_dor.sas</t>
+          <t>t_os_primary.sas</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -2494,17 +2482,17 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>T14.2.13</t>
+          <t>T14.2.16</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.13</t>
+          <t>Table 14.2.16</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Time to Response (TTR)</t>
+          <t>PFS — Sensitivity Analysis</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2519,7 +2507,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Responders (Confirmed CR or PR)</t>
+          <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2529,12 +2517,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADTTE</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>t_ttr.sas</t>
+          <t>t_pfs_sensitivity.sas</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -2553,17 +2541,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>T14.2.14</t>
+          <t>T14.2.17</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.14</t>
+          <t>Table 14.2.17</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Progression-Free Survival (PFS) — Primary Analysis</t>
+          <t>PFS — Subgroup Analysis</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2593,7 +2581,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>t_pfs_primary.sas</t>
+          <t>t_pfs_subgroup.sas</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -2612,17 +2600,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>T14.2.15</t>
+          <t>T14.2.18</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.15</t>
+          <t>Table 14.2.18</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Overall Survival (OS) — Primary Analysis</t>
+          <t>OS — Subgroup Analysis</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2652,7 +2640,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>t_os_primary.sas</t>
+          <t>t_os_subgroup.sas</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -2671,17 +2659,17 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>T14.2.16</t>
+          <t>T14.2.19</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.16</t>
+          <t>Table 14.2.19</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PFS — Sensitivity Analysis</t>
+          <t>Summary of Target Lesion Changes from Baseline</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2696,7 +2684,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>ITT with Measurable Disease and Post-Baseline Assessment</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2706,12 +2694,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADTTE</t>
+          <t>ADSL, ADRS</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>t_pfs_sensitivity.sas</t>
+          <t>t_target_lesion.sas</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -2730,17 +2718,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>T14.2.17</t>
+          <t>T14.2.20</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.17</t>
+          <t>Table 14.2.20</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>PFS — Subgroup Analysis</t>
+          <t>Landmark Analysis of OS by 6-Month PFS Status</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2755,7 +2743,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>ITT Alive and On-Study at 6 Months</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2770,7 +2758,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>t_pfs_subgroup.sas</t>
+          <t>t_landmark_os.sas</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -2789,17 +2777,17 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>T14.2.18</t>
+          <t>T14.2.21</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.18</t>
+          <t>Table 14.2.21</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>OS — Subgroup Analysis</t>
+          <t>Time to First Subsequent Therapy (TFST)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2814,7 +2802,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>ITT Population</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2824,12 +2812,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADTTE</t>
+          <t>ADSL, ADTTE, ADCM</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>t_os_subgroup.sas</t>
+          <t>t_tfst.sas</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -2848,17 +2836,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>T14.2.19</t>
+          <t>T14.2.22</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.19</t>
+          <t>Table 14.2.22</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Summary of Target Lesion Changes from Baseline</t>
+          <t>PK/PD Exposure-Response Correlation Analysis</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2873,22 +2861,22 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>ITT with Measurable Disease and Post-Baseline Assessment</t>
+          <t>PK/PD Evaluable Population</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Oncology only</t>
+          <t>General</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADPK, ADEFF</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>t_target_lesion.sas</t>
+          <t>t_pkpd_corr.sas</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -2905,137 +2893,145 @@
       <c r="M40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>T14.2.20</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.2.20</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Landmark Analysis of OS by 6-Month PFS Status</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>F14.2.1</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.2.1</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Forest Plot — Primary Endpoint by Subgroup</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>ITT Alive and On-Study at 6 Months</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Oncology only</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADTTE</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>t_landmark_os.sas</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Intent-to-Treat (ITT) Population</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADEFF</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>f_forest_primary.sas</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr"/>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>T14.2.21</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.2.21</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Time to First Subsequent Therapy (TFST)</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>F14.2.2</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.2.2</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Longitudinal Plot — Primary Endpoint Over Time</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>ITT Population</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Oncology only</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADTTE, ADCM</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>t_tfst.sas</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Intent-to-Treat (ITT) Population</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADEFF</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>f_longitudinal_eff.sas</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr"/>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>F14.2.4</t>
+          <t>F14.2.3</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.4</t>
+          <t>Figure 14.2.3</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Waterfall Plot — Best Percentage Change in Target Lesions</t>
+          <t>Cumulative Distribution Function Plot of Primary Endpoint</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -3050,22 +3046,22 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>ITT with Measurable Disease and Post-Baseline Assessment</t>
+          <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Oncology only</t>
+          <t>General</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADEFF</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>f_waterfall.sas</t>
+          <t>f_cdf_eff.sas</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr"/>
@@ -3088,17 +3084,17 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>F14.2.5</t>
+          <t>F14.2.4</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.5</t>
+          <t>Figure 14.2.4</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Spider Plot — Percentage Change in Tumor Burden Over Time</t>
+          <t>Waterfall Plot — Best Percentage Change in Target Lesions</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -3113,7 +3109,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>ITT with Measurable Disease</t>
+          <t>ITT with Measurable Disease and Post-Baseline Assessment</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -3128,7 +3124,7 @@
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>f_spider.sas</t>
+          <t>f_waterfall.sas</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr"/>
@@ -3151,17 +3147,17 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>F14.2.6</t>
+          <t>F14.2.5</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.6</t>
+          <t>Figure 14.2.5</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Swimmer Plot — Duration of Treatment and Response</t>
+          <t>Spider Plot — Percentage Change in Tumor Burden Over Time</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -3176,7 +3172,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Safety Population</t>
+          <t>ITT with Measurable Disease</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -3186,12 +3182,12 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>ADSL, ADEX, ADRS</t>
+          <t>ADSL, ADRS</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>f_swimmer.sas</t>
+          <t>f_spider.sas</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr"/>
@@ -3214,17 +3210,17 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>F14.2.7</t>
+          <t>F14.2.6</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.7</t>
+          <t>Figure 14.2.6</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Kaplan-Meier Plot — Progression-Free Survival</t>
+          <t>Swimmer Plot — Duration of Treatment and Response</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -3239,7 +3235,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>Safety Population</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -3249,12 +3245,12 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>ADSL, ADTTE</t>
+          <t>ADSL, ADEX, ADRS</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>f_km_pfs.sas</t>
+          <t>f_swimmer.sas</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr"/>
@@ -3277,17 +3273,17 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>F14.2.8</t>
+          <t>F14.2.7</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.8</t>
+          <t>Figure 14.2.7</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Kaplan-Meier Plot — Overall Survival</t>
+          <t>Kaplan-Meier Plot — Progression-Free Survival</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -3317,7 +3313,7 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>f_km_os.sas</t>
+          <t>f_km_pfs.sas</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr"/>
@@ -3340,17 +3336,17 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>F14.2.9</t>
+          <t>F14.2.8</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.9</t>
+          <t>Figure 14.2.8</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Forest Plot — PFS by Subgroup</t>
+          <t>Kaplan-Meier Plot — Overall Survival</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -3380,7 +3376,7 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>f_forest_pfs.sas</t>
+          <t>f_km_os.sas</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr"/>
@@ -3403,17 +3399,17 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>F14.2.10</t>
+          <t>F14.2.9</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.10</t>
+          <t>Figure 14.2.9</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Forest Plot — OS by Subgroup</t>
+          <t>Forest Plot — PFS by Subgroup</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -3443,7 +3439,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>f_forest_os.sas</t>
+          <t>f_forest_pfs.sas</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr"/>
@@ -3464,63 +3460,67 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>T14.2.22</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.2.22</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>PK/PD Exposure-Response Correlation Analysis</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>F14.2.10</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.2.10</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Forest Plot — OS by Subgroup</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>PK/PD Evaluable Population</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADPK, ADEFF</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>t_pkpd_corr.sas</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr"/>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M50" s="2" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Intent-to-Treat (ITT) Population</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Oncology only</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADTTE</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>f_forest_os.sas</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -9135,82 +9135,78 @@
       <c r="M142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
-      <c r="A143" s="3" t="inlineStr">
-        <is>
-          <t>F14.4.1</t>
-        </is>
-      </c>
-      <c r="B143" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.4.1</t>
-        </is>
-      </c>
-      <c r="C143" s="3" t="inlineStr">
-        <is>
-          <t>Pharmacokinetic (PK) Plot — Mean Serum Concentration-Time Profiles</t>
-        </is>
-      </c>
-      <c r="D143" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E143" s="3" t="inlineStr">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>T14.4.8</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.4.8</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>ADA Titer Distribution by Visit — Negative, Low, Medium, High</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
         <is>
           <t>14.4</t>
         </is>
       </c>
-      <c r="F143" s="3" t="inlineStr">
-        <is>
-          <t>PK Population</t>
-        </is>
-      </c>
-      <c r="G143" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H143" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADPC</t>
-        </is>
-      </c>
-      <c r="I143" s="3" t="inlineStr">
-        <is>
-          <t>f_pk_profile.sas</t>
-        </is>
-      </c>
-      <c r="J143" s="3" t="inlineStr"/>
-      <c r="K143" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L143" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M143" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Safety Population with ADA Samples</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADIS</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>t_ada_titer.sas</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr"/>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>T14.4.8</t>
+          <t>T14.4.9</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Table 14.4.8</t>
+          <t>Table 14.4.9</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>ADA Titer Distribution by Visit — Negative, Low, Medium, High</t>
+          <t>ADA Impact on Pharmacokinetics — Cmax and AUC in ADA+ vs. ADA- Subjects</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -9225,7 +9221,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>Safety Population with ADA Samples</t>
+          <t>PK Population with ADA Data</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -9235,12 +9231,12 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADIS</t>
+          <t>ADSL, ADIS, ADPP</t>
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>t_ada_titer.sas</t>
+          <t>t_ada_pk_impact.sas</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr"/>
@@ -9257,82 +9253,78 @@
       <c r="M144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
-      <c r="A145" s="3" t="inlineStr">
-        <is>
-          <t>F14.4.2</t>
-        </is>
-      </c>
-      <c r="B145" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.4.2</t>
-        </is>
-      </c>
-      <c r="C145" s="3" t="inlineStr">
-        <is>
-          <t>Overlaying Individual PK Concentration Profiles</t>
-        </is>
-      </c>
-      <c r="D145" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E145" s="3" t="inlineStr">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>T14.4.10</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.4.10</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Neutralizing Antibody (Nab) — Incidence, Titer, and Cross-Reactivity Status</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
         <is>
           <t>14.4</t>
         </is>
       </c>
-      <c r="F145" s="3" t="inlineStr">
-        <is>
-          <t>PK Population</t>
-        </is>
-      </c>
-      <c r="G145" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H145" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADPC</t>
-        </is>
-      </c>
-      <c r="I145" s="3" t="inlineStr">
-        <is>
-          <t>f_pk_overlay.sas</t>
-        </is>
-      </c>
-      <c r="J145" s="3" t="inlineStr"/>
-      <c r="K145" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L145" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M145" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Safety Population with ADA Samples</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADIS</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>t_nab_detail.sas</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr"/>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>T14.4.9</t>
+          <t>T14.4.11</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Table 14.4.9</t>
+          <t>Table 14.4.11</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>ADA Impact on Pharmacokinetics — Cmax and AUC in ADA+ vs. ADA- Subjects</t>
+          <t>Soluble Pharmacodynamic Biomarker Change from Baseline Over Time</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -9347,7 +9339,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>PK Population with ADA Data</t>
+          <t>PD Population</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -9357,12 +9349,12 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADIS, ADPP</t>
+          <t>ADSL, ADBM</t>
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>t_ada_pk_impact.sas</t>
+          <t>t_pd_bio_chg.sas</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr"/>
@@ -9379,82 +9371,78 @@
       <c r="M146" s="2" t="inlineStr"/>
     </row>
     <row r="147">
-      <c r="A147" s="3" t="inlineStr">
-        <is>
-          <t>F14.4.3</t>
-        </is>
-      </c>
-      <c r="B147" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.4.3</t>
-        </is>
-      </c>
-      <c r="C147" s="3" t="inlineStr">
-        <is>
-          <t>Mean (SD) Soluble EGFR and cMet Over Time</t>
-        </is>
-      </c>
-      <c r="D147" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E147" s="3" t="inlineStr">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>T14.4.12</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.4.12</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Trough PK Concentration (Ctrough) by Cycle — Target Attainment</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
         <is>
           <t>14.4</t>
         </is>
       </c>
-      <c r="F147" s="3" t="inlineStr">
-        <is>
-          <t>PD Population</t>
-        </is>
-      </c>
-      <c r="G147" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H147" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADPD</t>
-        </is>
-      </c>
-      <c r="I147" s="3" t="inlineStr">
-        <is>
-          <t>f_pd_time.sas</t>
-        </is>
-      </c>
-      <c r="J147" s="3" t="inlineStr"/>
-      <c r="K147" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L147" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M147" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>PK Population</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADPC</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>t_ctrough.sas</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr"/>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>T14.4.10</t>
+          <t>T14.4.13</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Table 14.4.10</t>
+          <t>Table 14.4.13</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Neutralizing Antibody (Nab) — Incidence, Titer, and Cross-Reactivity Status</t>
+          <t>Steady-State Attainment — Trough Concentrations Across Dosing Cycles (ANOVA)</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -9469,7 +9457,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>Safety Population with ADA Samples</t>
+          <t>PK Population</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -9479,12 +9467,12 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADIS</t>
+          <t>ADSL, ADPC</t>
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>t_nab_detail.sas</t>
+          <t>t_steady_state.sas</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr"/>
@@ -9501,303 +9489,315 @@
       <c r="M148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
-      <c r="A149" s="3" t="inlineStr">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>T14.4.14</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.4.14</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Urine Pharmacokinetic Parameters — Renal Excretion and Cumulative Recovery</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>PK Population (Subset with Urine PK)</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADPP</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>t_urine_pk.sas</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr"/>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>F14.4.1</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.4.1</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>Pharmacokinetic (PK) Plot — Mean Serum Concentration-Time Profiles</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>PK Population</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADPC</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
+          <t>f_pk_profile.sas</t>
+        </is>
+      </c>
+      <c r="J150" s="3" t="inlineStr"/>
+      <c r="K150" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L150" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M150" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>F14.4.2</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.4.2</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>Overlaying Individual PK Concentration Profiles</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>PK Population</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADPC</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="inlineStr">
+        <is>
+          <t>f_pk_overlay.sas</t>
+        </is>
+      </c>
+      <c r="J151" s="3" t="inlineStr"/>
+      <c r="K151" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L151" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M151" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>F14.4.3</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.4.3</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>Mean (SD) Soluble EGFR and cMet Over Time</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>PD Population</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADPD</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
+          <t>f_pd_time.sas</t>
+        </is>
+      </c>
+      <c r="J152" s="3" t="inlineStr"/>
+      <c r="K152" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L152" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M152" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
         <is>
           <t>F14.4.4</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B153" s="3" t="inlineStr">
         <is>
           <t>Figure 14.4.4</t>
         </is>
       </c>
-      <c r="C149" s="3" t="inlineStr">
+      <c r="C153" s="3" t="inlineStr">
         <is>
           <t>Boxplot of Biomarkers at Baseline vs. Response Status</t>
         </is>
       </c>
-      <c r="D149" s="3" t="inlineStr">
+      <c r="D153" s="3" t="inlineStr">
         <is>
           <t>Figure</t>
         </is>
       </c>
-      <c r="E149" s="3" t="inlineStr">
+      <c r="E153" s="3" t="inlineStr">
         <is>
           <t>14.4</t>
         </is>
       </c>
-      <c r="F149" s="3" t="inlineStr">
+      <c r="F153" s="3" t="inlineStr">
         <is>
           <t>Full Analysis Set with Biomarker Data</t>
         </is>
       </c>
-      <c r="G149" s="3" t="inlineStr">
+      <c r="G153" s="3" t="inlineStr">
         <is>
           <t>Oncology only</t>
         </is>
       </c>
-      <c r="H149" s="3" t="inlineStr">
+      <c r="H153" s="3" t="inlineStr">
         <is>
           <t>ADSL, ADBM</t>
         </is>
       </c>
-      <c r="I149" s="3" t="inlineStr">
+      <c r="I153" s="3" t="inlineStr">
         <is>
           <t>f_biomarker_box.sas</t>
         </is>
       </c>
-      <c r="J149" s="3" t="inlineStr"/>
-      <c r="K149" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L149" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M149" s="3" t="inlineStr">
+      <c r="J153" s="3" t="inlineStr"/>
+      <c r="K153" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L153" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M153" s="3" t="inlineStr">
         <is>
           <t>Simulated figure generated</t>
         </is>
       </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="2" t="inlineStr">
-        <is>
-          <t>T14.4.11</t>
-        </is>
-      </c>
-      <c r="B150" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.4.11</t>
-        </is>
-      </c>
-      <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>Soluble Pharmacodynamic Biomarker Change from Baseline Over Time</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E150" s="2" t="inlineStr">
-        <is>
-          <t>14.4</t>
-        </is>
-      </c>
-      <c r="F150" s="2" t="inlineStr">
-        <is>
-          <t>PD Population</t>
-        </is>
-      </c>
-      <c r="G150" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H150" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADBM</t>
-        </is>
-      </c>
-      <c r="I150" s="2" t="inlineStr">
-        <is>
-          <t>t_pd_bio_chg.sas</t>
-        </is>
-      </c>
-      <c r="J150" s="2" t="inlineStr"/>
-      <c r="K150" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L150" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M150" s="2" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
-        <is>
-          <t>T14.4.12</t>
-        </is>
-      </c>
-      <c r="B151" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.4.12</t>
-        </is>
-      </c>
-      <c r="C151" s="2" t="inlineStr">
-        <is>
-          <t>Trough PK Concentration (Ctrough) by Cycle — Target Attainment</t>
-        </is>
-      </c>
-      <c r="D151" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E151" s="2" t="inlineStr">
-        <is>
-          <t>14.4</t>
-        </is>
-      </c>
-      <c r="F151" s="2" t="inlineStr">
-        <is>
-          <t>PK Population</t>
-        </is>
-      </c>
-      <c r="G151" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H151" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADPC</t>
-        </is>
-      </c>
-      <c r="I151" s="2" t="inlineStr">
-        <is>
-          <t>t_ctrough.sas</t>
-        </is>
-      </c>
-      <c r="J151" s="2" t="inlineStr"/>
-      <c r="K151" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L151" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M151" s="2" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
-        <is>
-          <t>T14.4.13</t>
-        </is>
-      </c>
-      <c r="B152" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.4.13</t>
-        </is>
-      </c>
-      <c r="C152" s="2" t="inlineStr">
-        <is>
-          <t>Steady-State Attainment — Trough Concentrations Across Dosing Cycles (ANOVA)</t>
-        </is>
-      </c>
-      <c r="D152" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>14.4</t>
-        </is>
-      </c>
-      <c r="F152" s="2" t="inlineStr">
-        <is>
-          <t>PK Population</t>
-        </is>
-      </c>
-      <c r="G152" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H152" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADPC</t>
-        </is>
-      </c>
-      <c r="I152" s="2" t="inlineStr">
-        <is>
-          <t>t_steady_state.sas</t>
-        </is>
-      </c>
-      <c r="J152" s="2" t="inlineStr"/>
-      <c r="K152" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L152" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M152" s="2" t="inlineStr"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="2" t="inlineStr">
-        <is>
-          <t>T14.4.14</t>
-        </is>
-      </c>
-      <c r="B153" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.4.14</t>
-        </is>
-      </c>
-      <c r="C153" s="2" t="inlineStr">
-        <is>
-          <t>Urine Pharmacokinetic Parameters — Renal Excretion and Cumulative Recovery</t>
-        </is>
-      </c>
-      <c r="D153" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E153" s="2" t="inlineStr">
-        <is>
-          <t>14.4</t>
-        </is>
-      </c>
-      <c r="F153" s="2" t="inlineStr">
-        <is>
-          <t>PK Population (Subset with Urine PK)</t>
-        </is>
-      </c>
-      <c r="G153" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H153" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADPP</t>
-        </is>
-      </c>
-      <c r="I153" s="2" t="inlineStr">
-        <is>
-          <t>t_urine_pk.sas</t>
-        </is>
-      </c>
-      <c r="J153" s="2" t="inlineStr"/>
-      <c r="K153" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L153" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -13344,208 +13344,196 @@
       <c r="M9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>F14.2.1</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.2.1</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Forest Plot — Primary Endpoint by Subgroup</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>T14.2.9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.2.9</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Tumor Response — Best Overall Response (BOR)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADEFF</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>f_forest_primary.sas</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Oncology only</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADRS</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>t_bor.sas</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>F14.2.2</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.2.2</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Longitudinal Plot — Primary Endpoint Over Time</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>T14.2.10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.2.10</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Tumor Response — Objective Response Rate (ORR)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADEFF</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>f_longitudinal_eff.sas</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Oncology only</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADRS</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>t_orr.sas</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>F14.2.3</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.2.3</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Cumulative Distribution Function Plot of Primary Endpoint</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>T14.2.11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.2.11</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Tumor Response — Disease Control Rate (DCR)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADEFF</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>f_cdf_eff.sas</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Oncology only</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADRS</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>t_dcr.sas</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>T14.2.9</t>
+          <t>T14.2.12</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.9</t>
+          <t>Table 14.2.12</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Best Overall Response (BOR)</t>
+          <t>Tumor Response — Duration of Response (DOR)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -13560,7 +13548,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>Responders (Confirmed CR or PR)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -13570,12 +13558,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADRS, ADTTE</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>t_bor.sas</t>
+          <t>t_dor.sas</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
@@ -13594,17 +13582,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>T14.2.10</t>
+          <t>T14.2.13</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.10</t>
+          <t>Table 14.2.13</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Objective Response Rate (ORR)</t>
+          <t>Tumor Response — Time to Response (TTR)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -13619,7 +13607,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>Responders (Confirmed CR or PR)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -13634,7 +13622,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>t_orr.sas</t>
+          <t>t_ttr.sas</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
@@ -13653,17 +13641,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>T14.2.11</t>
+          <t>T14.2.14</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.11</t>
+          <t>Table 14.2.14</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Disease Control Rate (DCR)</t>
+          <t>Progression-Free Survival (PFS) — Primary Analysis</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -13688,12 +13676,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADTTE</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>t_dcr.sas</t>
+          <t>t_pfs_primary.sas</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
@@ -13712,17 +13700,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>T14.2.12</t>
+          <t>T14.2.15</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.12</t>
+          <t>Table 14.2.15</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Duration of Response (DOR)</t>
+          <t>Overall Survival (OS) — Primary Analysis</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -13737,7 +13725,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Responders (Confirmed CR or PR)</t>
+          <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -13747,12 +13735,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS, ADTTE</t>
+          <t>ADSL, ADTTE</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>t_dor.sas</t>
+          <t>t_os_primary.sas</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
@@ -13771,17 +13759,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>T14.2.13</t>
+          <t>T14.2.16</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.13</t>
+          <t>Table 14.2.16</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Tumor Response — Time to Response (TTR)</t>
+          <t>PFS — Sensitivity Analysis</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -13796,7 +13784,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Responders (Confirmed CR or PR)</t>
+          <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -13806,12 +13794,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADTTE</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>t_ttr.sas</t>
+          <t>t_pfs_sensitivity.sas</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
@@ -13830,17 +13818,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>T14.2.14</t>
+          <t>T14.2.17</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.14</t>
+          <t>Table 14.2.17</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Progression-Free Survival (PFS) — Primary Analysis</t>
+          <t>PFS — Subgroup Analysis</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -13870,7 +13858,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>t_pfs_primary.sas</t>
+          <t>t_pfs_subgroup.sas</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -13889,17 +13877,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>T14.2.15</t>
+          <t>T14.2.18</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.15</t>
+          <t>Table 14.2.18</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Overall Survival (OS) — Primary Analysis</t>
+          <t>OS — Subgroup Analysis</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -13929,7 +13917,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>t_os_primary.sas</t>
+          <t>t_os_subgroup.sas</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
@@ -13948,17 +13936,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>T14.2.16</t>
+          <t>T14.2.19</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.16</t>
+          <t>Table 14.2.19</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>PFS — Sensitivity Analysis</t>
+          <t>Summary of Target Lesion Changes from Baseline</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -13973,7 +13961,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>ITT with Measurable Disease and Post-Baseline Assessment</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -13983,12 +13971,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADTTE</t>
+          <t>ADSL, ADRS</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>t_pfs_sensitivity.sas</t>
+          <t>t_target_lesion.sas</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
@@ -14007,17 +13995,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>T14.2.17</t>
+          <t>T14.2.20</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.17</t>
+          <t>Table 14.2.20</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>PFS — Subgroup Analysis</t>
+          <t>Landmark Analysis of OS by 6-Month PFS Status</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -14032,7 +14020,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>ITT Alive and On-Study at 6 Months</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -14047,7 +14035,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>t_pfs_subgroup.sas</t>
+          <t>t_landmark_os.sas</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
@@ -14066,17 +14054,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>T14.2.18</t>
+          <t>T14.2.21</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.18</t>
+          <t>Table 14.2.21</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>OS — Subgroup Analysis</t>
+          <t>Time to First Subsequent Therapy (TFST)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -14091,7 +14079,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>ITT Population</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -14101,12 +14089,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADTTE</t>
+          <t>ADSL, ADTTE, ADCM</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>t_os_subgroup.sas</t>
+          <t>t_tfst.sas</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
@@ -14125,17 +14113,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>T14.2.19</t>
+          <t>T14.2.22</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Table 14.2.19</t>
+          <t>Table 14.2.22</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Summary of Target Lesion Changes from Baseline</t>
+          <t>PK/PD Exposure-Response Correlation Analysis</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -14150,22 +14138,22 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>ITT with Measurable Disease and Post-Baseline Assessment</t>
+          <t>PK/PD Evaluable Population</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Oncology only</t>
+          <t>General</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADPK, ADEFF</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>t_target_lesion.sas</t>
+          <t>t_pkpd_corr.sas</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr"/>
@@ -14182,137 +14170,145 @@
       <c r="M23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>T14.2.20</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.2.20</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Landmark Analysis of OS by 6-Month PFS Status</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>F14.2.1</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.2.1</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Forest Plot — Primary Endpoint by Subgroup</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>ITT Alive and On-Study at 6 Months</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Oncology only</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADTTE</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>t_landmark_os.sas</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Intent-to-Treat (ITT) Population</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADEFF</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>f_forest_primary.sas</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>T14.2.21</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.2.21</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Time to First Subsequent Therapy (TFST)</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>F14.2.2</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.2.2</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Longitudinal Plot — Primary Endpoint Over Time</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>ITT Population</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>Oncology only</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADTTE, ADCM</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>t_tfst.sas</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Intent-to-Treat (ITT) Population</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADEFF</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>f_longitudinal_eff.sas</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>F14.2.4</t>
+          <t>F14.2.3</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.4</t>
+          <t>Figure 14.2.3</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Waterfall Plot — Best Percentage Change in Target Lesions</t>
+          <t>Cumulative Distribution Function Plot of Primary Endpoint</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -14327,22 +14323,22 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>ITT with Measurable Disease and Post-Baseline Assessment</t>
+          <t>Intent-to-Treat (ITT) Population</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Oncology only</t>
+          <t>General</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>ADSL, ADRS</t>
+          <t>ADSL, ADEFF</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>f_waterfall.sas</t>
+          <t>f_cdf_eff.sas</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr"/>
@@ -14365,17 +14361,17 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>F14.2.5</t>
+          <t>F14.2.4</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.5</t>
+          <t>Figure 14.2.4</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Spider Plot — Percentage Change in Tumor Burden Over Time</t>
+          <t>Waterfall Plot — Best Percentage Change in Target Lesions</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -14390,7 +14386,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>ITT with Measurable Disease</t>
+          <t>ITT with Measurable Disease and Post-Baseline Assessment</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -14405,7 +14401,7 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>f_spider.sas</t>
+          <t>f_waterfall.sas</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr"/>
@@ -14428,17 +14424,17 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>F14.2.6</t>
+          <t>F14.2.5</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.6</t>
+          <t>Figure 14.2.5</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Swimmer Plot — Duration of Treatment and Response</t>
+          <t>Spider Plot — Percentage Change in Tumor Burden Over Time</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -14453,7 +14449,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Safety Population</t>
+          <t>ITT with Measurable Disease</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -14463,12 +14459,12 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>ADSL, ADEX, ADRS</t>
+          <t>ADSL, ADRS</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>f_swimmer.sas</t>
+          <t>f_spider.sas</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr"/>
@@ -14491,17 +14487,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>F14.2.7</t>
+          <t>F14.2.6</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.7</t>
+          <t>Figure 14.2.6</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Kaplan-Meier Plot — Progression-Free Survival</t>
+          <t>Swimmer Plot — Duration of Treatment and Response</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -14516,7 +14512,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Intent-to-Treat (ITT) Population</t>
+          <t>Safety Population</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -14526,12 +14522,12 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>ADSL, ADTTE</t>
+          <t>ADSL, ADEX, ADRS</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>f_km_pfs.sas</t>
+          <t>f_swimmer.sas</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr"/>
@@ -14554,17 +14550,17 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>F14.2.8</t>
+          <t>F14.2.7</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.8</t>
+          <t>Figure 14.2.7</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Kaplan-Meier Plot — Overall Survival</t>
+          <t>Kaplan-Meier Plot — Progression-Free Survival</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -14594,7 +14590,7 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>f_km_os.sas</t>
+          <t>f_km_pfs.sas</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr"/>
@@ -14617,17 +14613,17 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>F14.2.9</t>
+          <t>F14.2.8</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.9</t>
+          <t>Figure 14.2.8</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Forest Plot — PFS by Subgroup</t>
+          <t>Kaplan-Meier Plot — Overall Survival</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -14657,7 +14653,7 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>f_forest_pfs.sas</t>
+          <t>f_km_os.sas</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr"/>
@@ -14680,17 +14676,17 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>F14.2.10</t>
+          <t>F14.2.9</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Figure 14.2.10</t>
+          <t>Figure 14.2.9</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Forest Plot — OS by Subgroup</t>
+          <t>Forest Plot — PFS by Subgroup</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -14720,7 +14716,7 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>f_forest_os.sas</t>
+          <t>f_forest_pfs.sas</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr"/>
@@ -14741,63 +14737,67 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>T14.2.22</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.2.22</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>PK/PD Exposure-Response Correlation Analysis</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>F14.2.10</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.2.10</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Forest Plot — OS by Subgroup</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>14.2</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>PK/PD Evaluable Population</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADPK, ADEFF</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>t_pkpd_corr.sas</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Intent-to-Treat (ITT) Population</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Oncology only</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADTTE</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>f_forest_os.sas</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M33"/>
@@ -20608,82 +20608,78 @@
       <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>F14.4.1</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.4.1</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Pharmacokinetic (PK) Plot — Mean Serum Concentration-Time Profiles</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>T14.4.8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.4.8</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ADA Titer Distribution by Visit — Negative, Low, Medium, High</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>14.4</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>PK Population</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADPC</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>f_pk_profile.sas</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Safety Population with ADA Samples</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADIS</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>t_ada_titer.sas</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>T14.4.8</t>
+          <t>T14.4.9</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Table 14.4.8</t>
+          <t>Table 14.4.9</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ADA Titer Distribution by Visit — Negative, Low, Medium, High</t>
+          <t>ADA Impact on Pharmacokinetics — Cmax and AUC in ADA+ vs. ADA- Subjects</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -20698,7 +20694,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Safety Population with ADA Samples</t>
+          <t>PK Population with ADA Data</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -20708,12 +20704,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADIS</t>
+          <t>ADSL, ADIS, ADPP</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>t_ada_titer.sas</t>
+          <t>t_ada_pk_impact.sas</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
@@ -20730,82 +20726,78 @@
       <c r="M10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>F14.4.2</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.4.2</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Overlaying Individual PK Concentration Profiles</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>T14.4.10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.4.10</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Neutralizing Antibody (Nab) — Incidence, Titer, and Cross-Reactivity Status</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>14.4</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>PK Population</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADPC</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>f_pk_overlay.sas</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Safety Population with ADA Samples</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADIS</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>t_nab_detail.sas</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>T14.4.9</t>
+          <t>T14.4.11</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Table 14.4.9</t>
+          <t>Table 14.4.11</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>ADA Impact on Pharmacokinetics — Cmax and AUC in ADA+ vs. ADA- Subjects</t>
+          <t>Soluble Pharmacodynamic Biomarker Change from Baseline Over Time</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -20820,7 +20812,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>PK Population with ADA Data</t>
+          <t>PD Population</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -20830,12 +20822,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADIS, ADPP</t>
+          <t>ADSL, ADBM</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>t_ada_pk_impact.sas</t>
+          <t>t_pd_bio_chg.sas</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
@@ -20852,82 +20844,78 @@
       <c r="M12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>F14.4.3</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Figure 14.4.3</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Mean (SD) Soluble EGFR and cMet Over Time</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>T14.4.12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.4.12</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Trough PK Concentration (Ctrough) by Cycle — Target Attainment</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>14.4</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>PD Population</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>ADSL, ADPD</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>f_pd_time.sas</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Simulated figure generated</t>
-        </is>
-      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>PK Population</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADPC</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>t_ctrough.sas</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>T14.4.10</t>
+          <t>T14.4.13</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Table 14.4.10</t>
+          <t>Table 14.4.13</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Neutralizing Antibody (Nab) — Incidence, Titer, and Cross-Reactivity Status</t>
+          <t>Steady-State Attainment — Trough Concentrations Across Dosing Cycles (ANOVA)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -20942,7 +20930,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Safety Population with ADA Samples</t>
+          <t>PK Population</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -20952,12 +20940,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>ADSL, ADIS</t>
+          <t>ADSL, ADPC</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>t_nab_detail.sas</t>
+          <t>t_steady_state.sas</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
@@ -20974,303 +20962,315 @@
       <c r="M14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>T14.4.14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Table 14.4.14</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Urine Pharmacokinetic Parameters — Renal Excretion and Cumulative Recovery</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>PK Population (Subset with Urine PK)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>ADSL, ADPP</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>t_urine_pk.sas</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>F14.4.1</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.4.1</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Pharmacokinetic (PK) Plot — Mean Serum Concentration-Time Profiles</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>PK Population</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADPC</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>f_pk_profile.sas</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>F14.4.2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.4.2</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Overlaying Individual PK Concentration Profiles</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>PK Population</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADPC</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>f_pk_overlay.sas</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>F14.4.3</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Figure 14.4.3</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Mean (SD) Soluble EGFR and cMet Over Time</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>PD Population</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>ADSL, ADPD</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>f_pd_time.sas</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Simulated figure generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>F14.4.4</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Figure 14.4.4</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Boxplot of Biomarkers at Baseline vs. Response Status</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Figure</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>14.4</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Full Analysis Set with Biomarker Data</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Oncology only</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>ADSL, ADBM</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>f_biomarker_box.sas</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L15" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>First column retained; non-structural cells use XX</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>Simulated figure generated</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>T14.4.11</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.4.11</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Soluble Pharmacodynamic Biomarker Change from Baseline Over Time</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>14.4</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>PD Population</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADBM</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>t_pd_bio_chg.sas</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>T14.4.12</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.4.12</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Trough PK Concentration (Ctrough) by Cycle — Target Attainment</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>14.4</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>PK Population</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADPC</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>t_ctrough.sas</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>T14.4.13</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.4.13</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Steady-State Attainment — Trough Concentrations Across Dosing Cycles (ANOVA)</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>14.4</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>PK Population</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADPC</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>t_steady_state.sas</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>T14.4.14</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Table 14.4.14</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Urine Pharmacokinetic Parameters — Renal Excretion and Cumulative Recovery</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>14.4</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>PK Population (Subset with Urine PK)</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>ADSL, ADPP</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>t_urine_pk.sas</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>First column retained; non-structural cells use XX</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M19"/>
@@ -23663,7 +23663,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>27 April 2026</t>
+          <t>28 April 2026</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: Enhance TFLs-Shell Skill with Product Alignment Contracts and Validation
- Added output manifest and contract registry to define product-aligned outputs.
- Introduced new contracts for DOCX, XLSX, and SOP outputs, detailing structure and validation rules.
- Implemented scripts for exporting product contracts and validating outputs against defined contracts.
- Updated unit tests to cover new validation checks and ensure compliance with contracts.
- Created comprehensive documentation for catalog schema, DOCX shell, and output contracts.
- Established a process for maintaining contract integrity and preventing drift in product outputs.
</commit_message>
<xml_diff>
--- a/output/TFL_TOC_v2.1.0.xlsx
+++ b/output/TFL_TOC_v2.1.0.xlsx
@@ -32055,7 +32055,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Tables and listings preserve structural examples in the first column and use adaptive shell placeholders in non-structural cells. Expandable treatment/group patterns may include ellipsis (...) and a Total column, without concrete sample sizes in headers.</t>
+          <t>Tables and listings preserve structural examples in the first column and use adaptive shell placeholders in non-structural cells. Controlled treatment/group patterns use Group 1, Group 2, and may retain a separate ellipsis (...) expansion column; that expansion column must remain distinct and must not be merged with Overall, Total, HR, or other analytic columns. Header sample sizes remain generic rather than concrete.</t>
         </is>
       </c>
     </row>
@@ -32160,7 +32160,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>28 April 2026</t>
+          <t>29 April 2026</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: Update documentation and code to exclude Section 16.1 from scope across various components
</commit_message>
<xml_diff>
--- a/output/TFL_TOC_v2.1.0.xlsx
+++ b/output/TFL_TOC_v2.1.0.xlsx
@@ -32619,7 +32619,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>The workbook covers CSR Sections 14.1, 14.2, 14.3, 14.4, and 16.2 only; Section 16.1 is out of scope for this generator.</t>
+          <t>The workbook covers CSR Sections 14.1, 14.2, 14.3, 14.4, and 16.2.</t>
         </is>
       </c>
     </row>
@@ -32760,7 +32760,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>06 May 2026</t>
+          <t>07 May 2026</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add figure registry and mock data generation for shell rendering
- Implemented a new figure registry in `src/tflshell/figures/registry.py` to map figure types to their respective classes and generate mock data for rendering.
- Added functions to generate PNG buffers for figures and build mock data for various figure types including KM curves, waterfalls, spiders, swimmers, forests, box plots, and longitudinal data.
- Created unit tests for the figure rendering and catalog structure in `tests/unit/test_figure_shell_rendering.py` and `tests/unit/test_catalog_module_structure.py`.
- Added tests for section 14.1 in `tests/unit/test_section_14_1_practice.py` to ensure modular catalog slices and correct labeling of demographic characteristics.
</commit_message>
<xml_diff>
--- a/output/TFL_TOC_v2.1.0.xlsx
+++ b/output/TFL_TOC_v2.1.0.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Summary of Baseline Disease Characteristics</t>
+          <t>Summary of Baseline Oncology Disease Characteristics</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Oncology only</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Summary of Baseline Disease Characteristics</t>
+          <t>Summary of Baseline Oncology Disease Characteristics</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -16371,7 +16371,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Oncology only</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -32760,7 +32760,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>07 May 2026</t>
+          <t>17 June 2026</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">

</xml_diff>